<commit_message>
Stage 8 fixes: C-016
</commit_message>
<xml_diff>
--- a/output/archive/MerrivossData/Bioanalysis/AT15/MV-2015-240/MV-2015-240_AssayWorksheet_122115_v03.xlsx
+++ b/output/archive/MerrivossData/Bioanalysis/AT15/MV-2015-240/MV-2015-240_AssayWorksheet_122115_v03.xlsx
@@ -572,12 +572,17 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Compounds</t>
+          <t>Wider test article set</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
           <t>40</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Displayed PK subset: six compounds on Rat PK</t>
         </is>
       </c>
     </row>
@@ -757,7 +762,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sprague-Dawley rats, n = 3 per compound per route. IV at 1 mg/kg, PO at 5 mg/kg. CL in mL/min/kg, Vss in L/kg, F from the dose-normalised AUC ratio.</t>
+          <t>Displayed PK subset only: compounds identified below. Rat, 1 mg/kg IV and 5 mg/kg PO, n=3. CL in mL/min/kg, Vss in L/kg, F from dose-normalised AUC; do not extrapolate clearance/exposure to the wider set.</t>
         </is>
       </c>
     </row>
@@ -1032,22 +1037,22 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Blank plasma</t>
+          <t>Blank selectivity</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>No peak above LLOQ</t>
+          <t>Analyte-specific method/run acceptance sheets under M15/BIO/05540</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Study-plan limits: analyte interference relative to LLOQ; internal-standard interference relative to its response</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Accepted</t>
+          <t>Limits and observed responses are not reproduced; a blank below LLOQ does not establish selectivity.</t>
         </is>
       </c>
     </row>
@@ -1059,39 +1064,39 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Linear over the working range, r² above 0.99</t>
+          <t>Back-calculated concentrations and exclusions: original run acceptance sheets</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Method bias limits, LLOQ exception and minimum accepted calibrator proportion</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Accepted</t>
+          <t>Range and run identifiers remain in method/run records; no acceptance inferred from r².</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>QC samples</t>
+          <t>QC / failed-run disposition</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Within ±15% of nominal</t>
+          <t>Low-QC failure and repeat: run-disposition record under M15/BIO/05540</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Study-plan bias limits and minimum accepted proportions overall/per level</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Accepted; one low QC run repeated</t>
+          <t>Consult rejected-run and repeat identifiers, reason, sample reanalysis mapping and signed disposition; not transcribed here. Repeat not independently declared accepted.</t>
         </is>
       </c>
     </row>

</xml_diff>